<commit_message>
Block 3: Implementation + Execution
</commit_message>
<xml_diff>
--- a/results/block1_results/Normal_1/branches/dataframes/dataset_LCA_B02_Normal_1.xlsx
+++ b/results/block1_results/Normal_1/branches/dataframes/dataset_LCA_B02_Normal_1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I426"/>
+  <dimension ref="A1:J426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,6 +474,11 @@
           <t>PointType</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Segment_ID</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -509,6 +514,9 @@
           <t>Ostium</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -544,6 +552,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -579,6 +590,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -614,6 +628,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -649,6 +666,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -684,6 +704,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -719,6 +742,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -754,6 +780,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -789,6 +818,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -824,6 +856,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -859,6 +894,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -894,6 +932,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -929,6 +970,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -964,6 +1008,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -999,6 +1046,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J16" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1034,6 +1084,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J17" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1069,6 +1122,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1104,6 +1160,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J19" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1139,6 +1198,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1174,6 +1236,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J21" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1209,6 +1274,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J22" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1244,6 +1312,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J23" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1279,6 +1350,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1314,6 +1388,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J25" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1349,6 +1426,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J26" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1384,6 +1464,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J27" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1419,6 +1502,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J28" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1454,6 +1540,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J29" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1489,6 +1578,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J30" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1524,6 +1616,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J31" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1559,6 +1654,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J32" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1594,6 +1692,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J33" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1629,6 +1730,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J34" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1664,6 +1768,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J35" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1699,6 +1806,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J36" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1734,6 +1844,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J37" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1769,6 +1882,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J38" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1804,6 +1920,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J39" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1839,6 +1958,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J40" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1874,6 +1996,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J41" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1909,6 +2034,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J42" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1944,6 +2072,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J43" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1979,6 +2110,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J44" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2014,6 +2148,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J45" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2049,6 +2186,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J46" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2084,6 +2224,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J47" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2119,6 +2262,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J48" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2154,6 +2300,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J49" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2189,6 +2338,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J50" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2224,6 +2376,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J51" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -2259,6 +2414,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J52" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -2294,6 +2452,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J53" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -2329,6 +2490,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J54" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -2364,6 +2528,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J55" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2399,6 +2566,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J56" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2434,6 +2604,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J57" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -2469,6 +2642,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J58" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -2504,6 +2680,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J59" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -2539,6 +2718,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J60" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2574,6 +2756,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J61" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2609,6 +2794,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J62" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2644,6 +2832,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J63" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2679,6 +2870,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J64" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2714,6 +2908,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J65" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2749,6 +2946,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J66" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2784,6 +2984,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J67" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2819,6 +3022,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J68" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2854,6 +3060,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J69" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2889,6 +3098,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J70" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2924,6 +3136,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J71" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2959,6 +3174,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J72" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2994,6 +3212,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J73" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -3029,6 +3250,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J74" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -3064,6 +3288,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J75" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -3099,6 +3326,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J76" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -3134,6 +3364,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J77" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -3169,6 +3402,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J78" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3204,6 +3440,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J79" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -3239,6 +3478,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J80" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3274,6 +3516,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J81" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -3309,6 +3554,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J82" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -3344,6 +3592,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J83" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -3379,6 +3630,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J84" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -3414,6 +3668,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J85" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -3449,6 +3706,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J86" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3484,6 +3744,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J87" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3519,6 +3782,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J88" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3554,6 +3820,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J89" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3589,6 +3858,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J90" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3624,6 +3896,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J91" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3659,6 +3934,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J92" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3694,6 +3972,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J93" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3729,6 +4010,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J94" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -3764,6 +4048,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J95" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3799,6 +4086,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J96" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3834,6 +4124,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J97" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3869,6 +4162,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J98" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3904,6 +4200,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J99" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3939,6 +4238,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J100" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3974,6 +4276,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J101" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -4009,6 +4314,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J102" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -4044,6 +4352,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J103" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -4079,6 +4390,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J104" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -4114,6 +4428,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J105" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -4149,6 +4466,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J106" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -4184,6 +4504,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J107" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -4219,6 +4542,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J108" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -4254,6 +4580,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J109" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -4289,6 +4618,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J110" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4324,6 +4656,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J111" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -4359,6 +4694,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J112" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -4394,6 +4732,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J113" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -4429,6 +4770,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J114" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -4464,6 +4808,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J115" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4499,6 +4846,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J116" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4534,6 +4884,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J117" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -4569,6 +4922,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J118" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4604,6 +4960,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J119" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -4639,6 +4998,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J120" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -4674,6 +5036,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J121" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -4709,6 +5074,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J122" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -4744,6 +5112,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J123" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -4779,6 +5150,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J124" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -4814,6 +5188,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J125" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -4849,6 +5226,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J126" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -4884,6 +5264,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J127" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -4919,6 +5302,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J128" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -4954,6 +5340,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J129" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4989,6 +5378,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J130" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -5024,6 +5416,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J131" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -5059,6 +5454,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J132" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -5094,6 +5492,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J133" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -5129,6 +5530,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J134" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -5164,6 +5568,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J135" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -5199,6 +5606,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J136" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -5234,6 +5644,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J137" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -5269,6 +5682,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J138" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -5304,6 +5720,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J139" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -5339,6 +5758,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J140" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -5374,6 +5796,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J141" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -5409,6 +5834,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J142" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -5444,6 +5872,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J143" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -5479,6 +5910,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J144" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -5514,6 +5948,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J145" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -5549,6 +5986,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J146" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -5584,6 +6024,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J147" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -5619,6 +6062,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J148" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -5654,6 +6100,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J149" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -5689,6 +6138,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J150" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -5724,6 +6176,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J151" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -5759,6 +6214,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J152" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -5794,6 +6252,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J153" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -5829,6 +6290,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J154" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -5864,6 +6328,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J155" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -5899,6 +6366,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J156" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -5934,6 +6404,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J157" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -5969,6 +6442,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J158" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -6004,6 +6480,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J159" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -6039,6 +6518,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J160" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -6074,6 +6556,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J161" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -6109,6 +6594,9 @@
           <t>Bifurcation</t>
         </is>
       </c>
+      <c r="J162" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -6144,6 +6632,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J163" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -6179,6 +6670,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J164" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -6214,6 +6708,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J165" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -6249,6 +6746,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J166" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -6284,6 +6784,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J167" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -6319,6 +6822,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J168" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -6354,6 +6860,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J169" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -6389,6 +6898,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J170" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -6424,6 +6936,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J171" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -6459,6 +6974,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J172" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -6494,6 +7012,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J173" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -6529,6 +7050,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J174" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -6564,6 +7088,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J175" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -6599,6 +7126,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J176" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -6634,6 +7164,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J177" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -6669,6 +7202,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J178" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -6704,6 +7240,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J179" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -6739,6 +7278,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J180" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -6774,6 +7316,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J181" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -6809,6 +7354,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J182" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -6844,6 +7392,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J183" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -6879,6 +7430,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J184" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -6914,6 +7468,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J185" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -6949,6 +7506,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J186" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -6984,6 +7544,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J187" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -7019,6 +7582,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J188" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -7054,6 +7620,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J189" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -7089,6 +7658,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J190" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -7124,6 +7696,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J191" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -7159,6 +7734,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J192" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -7194,6 +7772,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J193" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -7229,6 +7810,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J194" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -7264,6 +7848,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J195" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -7299,6 +7886,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J196" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -7334,6 +7924,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J197" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -7369,6 +7962,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J198" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -7404,6 +8000,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J199" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -7439,6 +8038,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J200" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -7474,6 +8076,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J201" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
@@ -7509,6 +8114,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J202" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
@@ -7544,6 +8152,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J203" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
@@ -7579,6 +8190,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J204" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
@@ -7614,6 +8228,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J205" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
@@ -7649,6 +8266,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J206" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
@@ -7684,6 +8304,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J207" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
@@ -7719,6 +8342,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J208" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
@@ -7754,6 +8380,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J209" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
@@ -7789,6 +8418,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J210" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -7824,6 +8456,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J211" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
@@ -7859,6 +8494,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J212" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -7894,6 +8532,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J213" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
@@ -7929,6 +8570,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J214" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -7964,6 +8608,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J215" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -7999,6 +8646,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J216" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
@@ -8034,6 +8684,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J217" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="n">
@@ -8069,6 +8722,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J218" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="n">
@@ -8104,6 +8760,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J219" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="n">
@@ -8139,6 +8798,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J220" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
@@ -8174,6 +8836,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J221" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="n">
@@ -8209,6 +8874,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J222" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="n">
@@ -8244,6 +8912,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J223" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="n">
@@ -8279,6 +8950,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J224" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="n">
@@ -8314,6 +8988,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J225" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="n">
@@ -8349,6 +9026,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J226" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
@@ -8384,6 +9064,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J227" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
@@ -8419,6 +9102,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J228" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
@@ -8454,6 +9140,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J229" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
@@ -8489,6 +9178,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J230" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
@@ -8524,6 +9216,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J231" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
@@ -8559,6 +9254,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J232" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
@@ -8594,6 +9292,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J233" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
@@ -8629,6 +9330,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J234" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
@@ -8664,6 +9368,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J235" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
@@ -8699,6 +9406,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J236" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
@@ -8734,6 +9444,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J237" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
@@ -8769,6 +9482,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J238" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
@@ -8804,6 +9520,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J239" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="n">
@@ -8839,6 +9558,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J240" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="n">
@@ -8874,6 +9596,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J241" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="n">
@@ -8909,6 +9634,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J242" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="n">
@@ -8944,6 +9672,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J243" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="n">
@@ -8979,6 +9710,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J244" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="n">
@@ -9014,6 +9748,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J245" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="n">
@@ -9049,6 +9786,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J246" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="n">
@@ -9084,6 +9824,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J247" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="n">
@@ -9119,6 +9862,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J248" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="n">
@@ -9154,6 +9900,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J249" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="n">
@@ -9189,6 +9938,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J250" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="n">
@@ -9224,6 +9976,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J251" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="n">
@@ -9259,6 +10014,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J252" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="n">
@@ -9294,6 +10052,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J253" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="n">
@@ -9329,6 +10090,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J254" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -9364,6 +10128,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J255" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
@@ -9399,6 +10166,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J256" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -9434,6 +10204,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J257" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="n">
@@ -9469,6 +10242,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J258" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="n">
@@ -9504,6 +10280,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J259" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="n">
@@ -9539,6 +10318,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J260" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="n">
@@ -9574,6 +10356,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J261" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="n">
@@ -9609,6 +10394,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J262" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="n">
@@ -9644,6 +10432,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J263" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="n">
@@ -9679,6 +10470,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J264" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="n">
@@ -9714,6 +10508,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J265" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="n">
@@ -9749,6 +10546,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J266" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="n">
@@ -9784,6 +10584,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J267" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="n">
@@ -9819,6 +10622,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J268" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="n">
@@ -9854,6 +10660,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J269" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="n">
@@ -9889,6 +10698,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J270" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="n">
@@ -9924,6 +10736,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J271" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="n">
@@ -9959,6 +10774,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J272" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -9994,6 +10812,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J273" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="n">
@@ -10029,6 +10850,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J274" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="n">
@@ -10064,6 +10888,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J275" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -10099,6 +10926,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J276" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -10134,6 +10964,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J277" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="n">
@@ -10169,6 +11002,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J278" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -10204,6 +11040,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J279" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="n">
@@ -10239,6 +11078,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J280" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="n">
@@ -10274,6 +11116,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J281" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="n">
@@ -10309,6 +11154,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J282" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="n">
@@ -10344,6 +11192,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J283" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="n">
@@ -10379,6 +11230,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J284" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="n">
@@ -10414,6 +11268,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J285" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="n">
@@ -10449,6 +11306,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J286" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="n">
@@ -10484,6 +11344,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J287" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -10519,6 +11382,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J288" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="n">
@@ -10554,6 +11420,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J289" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="n">
@@ -10589,6 +11458,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J290" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -10624,6 +11496,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J291" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="n">
@@ -10659,6 +11534,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J292" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="n">
@@ -10694,6 +11572,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J293" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -10729,6 +11610,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J294" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="n">
@@ -10764,6 +11648,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J295" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="n">
@@ -10799,6 +11686,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J296" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="n">
@@ -10834,6 +11724,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J297" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="n">
@@ -10869,6 +11762,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J298" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="n">
@@ -10904,6 +11800,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J299" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="n">
@@ -10939,6 +11838,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J300" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="n">
@@ -10974,6 +11876,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J301" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="n">
@@ -11009,6 +11914,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J302" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="n">
@@ -11044,6 +11952,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J303" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="n">
@@ -11079,6 +11990,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J304" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="n">
@@ -11114,6 +12028,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J305" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -11149,6 +12066,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J306" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="n">
@@ -11184,6 +12104,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J307" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="n">
@@ -11219,6 +12142,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J308" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="309">
       <c r="A309" t="n">
@@ -11254,6 +12180,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J309" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="n">
@@ -11289,6 +12218,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J310" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="n">
@@ -11324,6 +12256,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J311" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -11359,6 +12294,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J312" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -11394,6 +12332,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J313" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -11429,6 +12370,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J314" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -11464,6 +12408,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J315" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="n">
@@ -11499,6 +12446,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J316" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="n">
@@ -11534,6 +12484,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J317" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="n">
@@ -11569,6 +12522,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J318" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="n">
@@ -11604,6 +12560,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J319" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="n">
@@ -11639,6 +12598,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J320" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="n">
@@ -11674,6 +12636,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J321" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="n">
@@ -11709,6 +12674,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J322" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="n">
@@ -11744,6 +12712,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J323" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="n">
@@ -11779,6 +12750,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J324" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="n">
@@ -11814,6 +12788,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J325" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="n">
@@ -11849,6 +12826,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J326" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="n">
@@ -11884,6 +12864,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J327" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="n">
@@ -11919,6 +12902,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J328" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="n">
@@ -11954,6 +12940,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J329" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="n">
@@ -11989,6 +12978,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J330" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="n">
@@ -12024,6 +13016,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J331" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="n">
@@ -12059,6 +13054,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J332" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="333">
       <c r="A333" t="n">
@@ -12094,6 +13092,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J333" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="n">
@@ -12129,6 +13130,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J334" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="n">
@@ -12164,6 +13168,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J335" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -12199,6 +13206,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J336" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="n">
@@ -12234,6 +13244,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J337" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -12269,6 +13282,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J338" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="n">
@@ -12304,6 +13320,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J339" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="n">
@@ -12339,6 +13358,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J340" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="n">
@@ -12374,6 +13396,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J341" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -12409,6 +13434,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J342" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="n">
@@ -12444,6 +13472,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J343" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="n">
@@ -12479,6 +13510,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J344" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="n">
@@ -12514,6 +13548,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J345" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="n">
@@ -12549,6 +13586,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J346" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="347">
       <c r="A347" t="n">
@@ -12584,6 +13624,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J347" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="n">
@@ -12619,6 +13662,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J348" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="n">
@@ -12654,6 +13700,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J349" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="n">
@@ -12689,6 +13738,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J350" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="n">
@@ -12724,6 +13776,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J351" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="n">
@@ -12759,6 +13814,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J352" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="353">
       <c r="A353" t="n">
@@ -12794,6 +13852,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J353" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="354">
       <c r="A354" t="n">
@@ -12829,6 +13890,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J354" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -12864,6 +13928,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J355" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="n">
@@ -12899,6 +13966,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J356" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="n">
@@ -12934,6 +14004,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J357" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="n">
@@ -12969,6 +14042,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J358" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="n">
@@ -13004,6 +14080,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J359" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="360">
       <c r="A360" t="n">
@@ -13039,6 +14118,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J360" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="n">
@@ -13074,6 +14156,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J361" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="n">
@@ -13109,6 +14194,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J362" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="363">
       <c r="A363" t="n">
@@ -13144,6 +14232,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J363" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="364">
       <c r="A364" t="n">
@@ -13179,6 +14270,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J364" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="365">
       <c r="A365" t="n">
@@ -13214,6 +14308,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J365" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -13249,6 +14346,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J366" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="367">
       <c r="A367" t="n">
@@ -13284,6 +14384,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J367" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="368">
       <c r="A368" t="n">
@@ -13319,6 +14422,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J368" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -13354,6 +14460,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J369" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="370">
       <c r="A370" t="n">
@@ -13389,6 +14498,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J370" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="371">
       <c r="A371" t="n">
@@ -13424,6 +14536,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J371" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="372">
       <c r="A372" t="n">
@@ -13459,6 +14574,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J372" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="373">
       <c r="A373" t="n">
@@ -13494,6 +14612,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J373" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="374">
       <c r="A374" t="n">
@@ -13529,6 +14650,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J374" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="375">
       <c r="A375" t="n">
@@ -13564,6 +14688,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J375" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="376">
       <c r="A376" t="n">
@@ -13599,6 +14726,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J376" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -13634,6 +14764,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J377" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="378">
       <c r="A378" t="n">
@@ -13669,6 +14802,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J378" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="379">
       <c r="A379" t="n">
@@ -13704,6 +14840,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J379" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -13739,6 +14878,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J380" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="381">
       <c r="A381" t="n">
@@ -13774,6 +14916,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J381" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="382">
       <c r="A382" t="n">
@@ -13809,6 +14954,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J382" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="383">
       <c r="A383" t="n">
@@ -13844,6 +14992,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J383" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="384">
       <c r="A384" t="n">
@@ -13879,6 +15030,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J384" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="385">
       <c r="A385" t="n">
@@ -13914,6 +15068,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J385" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="386">
       <c r="A386" t="n">
@@ -13949,6 +15106,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J386" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -13984,6 +15144,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J387" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="388">
       <c r="A388" t="n">
@@ -14019,6 +15182,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J388" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="389">
       <c r="A389" t="n">
@@ -14054,6 +15220,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J389" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="390">
       <c r="A390" t="n">
@@ -14089,6 +15258,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J390" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="391">
       <c r="A391" t="n">
@@ -14124,6 +15296,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J391" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" t="n">
@@ -14159,6 +15334,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J392" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" t="n">
@@ -14194,6 +15372,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J393" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" t="n">
@@ -14229,6 +15410,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J394" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -14264,6 +15448,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J395" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" t="n">
@@ -14299,6 +15486,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J396" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" t="n">
@@ -14334,6 +15524,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J397" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" t="n">
@@ -14369,6 +15562,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J398" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" t="n">
@@ -14404,6 +15600,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J399" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" t="n">
@@ -14439,6 +15638,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J400" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" t="n">
@@ -14474,6 +15676,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J401" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" t="n">
@@ -14509,6 +15714,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J402" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" t="n">
@@ -14544,6 +15752,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J403" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" t="n">
@@ -14579,6 +15790,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J404" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -14614,6 +15828,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J405" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" t="n">
@@ -14649,6 +15866,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J406" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" t="n">
@@ -14684,6 +15904,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J407" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" t="n">
@@ -14719,6 +15942,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J408" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" t="n">
@@ -14754,6 +15980,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J409" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" t="n">
@@ -14789,6 +16018,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J410" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" t="n">
@@ -14824,6 +16056,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J411" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" t="n">
@@ -14859,6 +16094,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J412" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" t="n">
@@ -14894,6 +16132,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J413" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" t="n">
@@ -14929,6 +16170,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J414" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" t="n">
@@ -14964,6 +16208,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J415" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" t="n">
@@ -14999,6 +16246,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J416" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" t="n">
@@ -15034,6 +16284,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J417" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="418">
       <c r="A418" t="n">
@@ -15069,6 +16322,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J418" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" t="n">
@@ -15104,6 +16360,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J419" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" t="n">
@@ -15139,6 +16398,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J420" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" t="n">
@@ -15174,6 +16436,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J421" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="422">
       <c r="A422" t="n">
@@ -15209,6 +16474,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J422" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="423">
       <c r="A423" t="n">
@@ -15244,6 +16512,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J423" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="424">
       <c r="A424" t="n">
@@ -15279,6 +16550,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J424" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="425">
       <c r="A425" t="n">
@@ -15314,6 +16588,9 @@
           <t>Standard</t>
         </is>
       </c>
+      <c r="J425" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="426">
       <c r="A426" t="n">
@@ -15348,6 +16625,9 @@
         <is>
           <t>Endpoint</t>
         </is>
+      </c>
+      <c r="J426" t="n">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>